<commit_message>
Aggiornamento data json e checklist
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#CENTROBIOLABSERVICE/CENTRO_BIOLAB_SERVICE_SRL/CBS_POLIAMBULATORIO/1.57/report-checklist.xlsx
+++ b/GATEWAY/A1#111#CENTROBIOLABSERVICE/CENTRO_BIOLAB_SERVICE_SRL/CBS_POLIAMBULATORIO/1.57/report-checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paolo\OneDrive\Desktop\FSE Puglia\accreditamento fse git\ESITO TESTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EEE4B4F-9328-462F-9093-F1F8AB7A4B65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0FD102C-3170-475C-A502-0659C7FD1BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1518" uniqueCount="546">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="547">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -1274,24 +1274,6 @@
     <t>L'invio al gateway è asincrono per permettere al medico di proseguire con la propria attività clinica. Sia il medico che il backoffice hanno a disposizione un cruscotto che mostra i messaggi non andati a buon fine con la descrizione dell'errore. Una volta che l'errore è stato corretto dal medico, in maniera autonoma o su segnalazione del backoffice, il documento rientra nella coda di firma e di ritrasmissione verso il gateway.</t>
   </si>
   <si>
-    <t>2026-03-17T10:39:30Z</t>
-  </si>
-  <si>
-    <t>6460c0149b6d4f9622adecd7ed7cd913</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.2b15007562^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-17T10:43:05Z</t>
-  </si>
-  <si>
-    <t>28142b9ace1546029827b80c15ac6d60</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.0a9151b717^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-03-17T18:19:17Z</t>
   </si>
   <si>
@@ -1472,24 +1454,6 @@
     <t>2.16.840.1.113883.2.9.2.120.4.4.8fe46b71d98546dc779f4a7f4859b056b254bbe56b59baa550333b2c46441c87.6e53c525a4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>2026-03-18T09:54:22Z</t>
-  </si>
-  <si>
-    <t>4c78cec009a930104f23195161c74056</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.8fe46b71d98546dc779f4a7f4859b056b254bbe56b59baa550333b2c46441c87.bba1279e31^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-18T10:07:57Z</t>
-  </si>
-  <si>
-    <t>622ee4a842d7096d1ceb65d4b2726c41</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.8fe46b71d98546dc779f4a7f4859b056b254bbe56b59baa550333b2c46441c87.5cb6736eb9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-03-18T12:48:57Z</t>
   </si>
   <si>
@@ -1571,24 +1535,6 @@
     <t>2.16.840.1.113883.2.9.2.120.4.4.97bb3fc5bee3032679f4f07419e04af6375baafa17024527a98ede920c6812ed.17bfae19f5^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>2026-03-18T16:19:03Z</t>
-  </si>
-  <si>
-    <t>114a92711423f74a2b36a0f73ac99eda</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.97bb3fc5bee3032679f4f07419e04af6375baafa17024527a98ede920c6812ed.6fe576f196^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-18T16:26:26Z</t>
-  </si>
-  <si>
-    <t>63782e109003b9114e3bcf931a0b26d8</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.97bb3fc5bee3032679f4f07419e04af6375baafa17024527a98ede920c6812ed.0de3add05d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-03-18T18:24:29Z</t>
   </si>
   <si>
@@ -1613,12 +1559,6 @@
     <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.760b449db6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>00b518b36e840ae0507c031ab4e66acc</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.44b5070a01^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-03-19T11:09:35Z</t>
   </si>
   <si>
@@ -1848,27 +1788,6 @@
   </si>
   <si>
     <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.e9f7a6768c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-18T18:57:34Z</t>
-  </si>
-  <si>
-    <t>2026-03-19T12:55:06Z</t>
-  </si>
-  <si>
-    <t>1305443d00aca2bf7145b91c70bb6347</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.75ac494b89^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-19T15:28:44Z</t>
-  </si>
-  <si>
-    <t>4722703084d03b3a4f91985f940efad5</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.aac0ebab71^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>2026-03-19T16:22:31Z</t>
@@ -2004,6 +1923,90 @@
   </si>
   <si>
     <t>Non Gestiamo Laboratori di Analisi che effettuano Trasfusioni</t>
+  </si>
+  <si>
+    <t>ddfbfc83a57d5ced3e759b90270940b6</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.c4a19ab08d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.be20a15514^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>704f665ed66c5cbcd6df451b38e22efa</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.8fe46b71d98546dc779f4a7f4859b056b254bbe56b59baa550333b2c46441c87.8ec86adcd6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>52e94d7170f4b0182ad993cf69b9f173</t>
+  </si>
+  <si>
+    <t>39fc441612ab744470c1ad3026939989</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.8fe46b71d98546dc779f4a7f4859b056b254bbe56b59baa550333b2c46441c87.0c9feae58a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T18:02:22Z</t>
+  </si>
+  <si>
+    <t>2026-03-30T18:25:58Z</t>
+  </si>
+  <si>
+    <t>2026-03-30T18:29:21Z</t>
+  </si>
+  <si>
+    <t>2026-03-30T18:32:37Z</t>
+  </si>
+  <si>
+    <t>2026-03-30T16:19:03Z</t>
+  </si>
+  <si>
+    <t>c9ac14d91a6521994e0e5e2d17787d56</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.97bb3fc5bee3032679f4f07419e04af6375baafa17024527a98ede920c6812ed.7402ea81d8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>ca5a49210d49663ee4e2b46baf363443</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.97bb3fc5bee3032679f4f07419e04af6375baafa17024527a98ede920c6812ed.778f52725e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-31T08:46:27Z</t>
+  </si>
+  <si>
+    <t>9b0b68160dafc70938db708407790326</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.40d0883912^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>31/03/2026</t>
+  </si>
+  <si>
+    <t>2026-03-31T09:03:46Z</t>
+  </si>
+  <si>
+    <t>2026-03-31T08:59:56Z</t>
+  </si>
+  <si>
+    <t>804c39bdfb45649a7a0198638da4fa2a</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.8ea47d33ac^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-31T09:08:30Z</t>
+  </si>
+  <si>
+    <t>e2ac9ee378eed70710d429e673992b50</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.b5ff942f15^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -2185,7 +2188,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="48">
+  <borders count="47">
     <border>
       <left/>
       <right/>
@@ -2634,21 +2637,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -2775,7 +2763,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2960,6 +2948,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2972,34 +2963,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3016,28 +3001,6 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -3069,17 +3032,33 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="47" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="47" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -4568,14 +4547,14 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="98" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="88"/>
-      <c r="C2" s="89" t="s">
+      <c r="B2" s="99"/>
+      <c r="C2" s="100" t="s">
         <v>267</v>
       </c>
-      <c r="D2" s="88"/>
+      <c r="D2" s="99"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -4596,14 +4575,14 @@
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="90" t="s">
+      <c r="A3" s="101" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="91"/>
-      <c r="C3" s="96" t="s">
+      <c r="B3" s="102"/>
+      <c r="C3" s="107" t="s">
         <v>268</v>
       </c>
-      <c r="D3" s="88"/>
+      <c r="D3" s="99"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -4624,12 +4603,12 @@
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="92"/>
-      <c r="B4" s="93"/>
-      <c r="C4" s="96" t="s">
+      <c r="A4" s="103"/>
+      <c r="B4" s="104"/>
+      <c r="C4" s="107" t="s">
         <v>269</v>
       </c>
-      <c r="D4" s="88"/>
+      <c r="D4" s="99"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -4651,12 +4630,12 @@
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="94"/>
-      <c r="B5" s="95"/>
-      <c r="C5" s="96" t="s">
+      <c r="A5" s="105"/>
+      <c r="B5" s="106"/>
+      <c r="C5" s="107" t="s">
         <v>270</v>
       </c>
-      <c r="D5" s="88"/>
+      <c r="D5" s="99"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -4677,8 +4656,8 @@
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="85"/>
-      <c r="B6" s="86"/>
+      <c r="A6" s="96"/>
+      <c r="B6" s="97"/>
       <c r="C6" s="10"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -4829,30 +4808,30 @@
       <c r="E10" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="77">
-        <v>46099</v>
-      </c>
-      <c r="G10" s="78" t="s">
-        <v>419</v>
-      </c>
-      <c r="H10" s="78" t="s">
-        <v>420</v>
-      </c>
-      <c r="I10" s="78" t="s">
-        <v>421</v>
-      </c>
-      <c r="J10" s="80" t="s">
-        <v>67</v>
-      </c>
-      <c r="K10" s="75"/>
+      <c r="F10" s="76">
+        <v>46112</v>
+      </c>
+      <c r="G10" s="77" t="s">
+        <v>536</v>
+      </c>
+      <c r="H10" s="77" t="s">
+        <v>534</v>
+      </c>
+      <c r="I10" s="77" t="s">
+        <v>535</v>
+      </c>
+      <c r="J10" s="79" t="s">
+        <v>67</v>
+      </c>
+      <c r="K10" s="74"/>
       <c r="L10" s="33"/>
-      <c r="M10" s="101"/>
-      <c r="N10" s="101"/>
-      <c r="O10" s="101"/>
+      <c r="M10" s="88"/>
+      <c r="N10" s="88"/>
+      <c r="O10" s="88"/>
       <c r="P10" s="43"/>
-      <c r="Q10" s="101"/>
-      <c r="R10" s="101"/>
-      <c r="S10" s="101"/>
+      <c r="Q10" s="88"/>
+      <c r="R10" s="88"/>
+      <c r="S10" s="88"/>
       <c r="T10" s="33"/>
       <c r="U10" s="34"/>
       <c r="V10" s="35"/>
@@ -4873,49 +4852,49 @@
       <c r="D11" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="100" t="s">
-        <v>521</v>
-      </c>
-      <c r="F11" s="99" t="s">
-        <v>520</v>
+      <c r="E11" s="87" t="s">
+        <v>494</v>
+      </c>
+      <c r="F11" s="86" t="s">
+        <v>493</v>
       </c>
       <c r="G11" s="50" t="s">
-        <v>525</v>
+        <v>498</v>
       </c>
       <c r="H11" s="50" t="s">
-        <v>522</v>
-      </c>
-      <c r="I11" s="76" t="s">
-        <v>523</v>
-      </c>
-      <c r="J11" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="K11" s="101"/>
-      <c r="L11" s="101"/>
-      <c r="M11" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="N11" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="O11" s="101"/>
+        <v>495</v>
+      </c>
+      <c r="I11" s="75" t="s">
+        <v>496</v>
+      </c>
+      <c r="J11" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="K11" s="88"/>
+      <c r="L11" s="88"/>
+      <c r="M11" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="N11" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="O11" s="88"/>
       <c r="P11" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="Q11" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="R11" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S11" s="101" t="s">
-        <v>543</v>
-      </c>
-      <c r="T11" s="101"/>
-      <c r="U11" s="102"/>
-      <c r="V11" s="103"/>
-      <c r="W11" s="104" t="s">
+      <c r="Q11" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="R11" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S11" s="88" t="s">
+        <v>516</v>
+      </c>
+      <c r="T11" s="88"/>
+      <c r="U11" s="89"/>
+      <c r="V11" s="90"/>
+      <c r="W11" s="91" t="s">
         <v>50</v>
       </c>
     </row>
@@ -4935,46 +4914,46 @@
       <c r="E12" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="F12" s="99" t="s">
-        <v>520</v>
+      <c r="F12" s="86" t="s">
+        <v>493</v>
       </c>
       <c r="G12" s="32" t="s">
-        <v>527</v>
+        <v>500</v>
       </c>
       <c r="H12" s="32" t="s">
-        <v>528</v>
+        <v>501</v>
       </c>
       <c r="I12" s="37" t="s">
-        <v>523</v>
-      </c>
-      <c r="J12" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="K12" s="101"/>
-      <c r="L12" s="101"/>
-      <c r="M12" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="N12" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="O12" s="101"/>
+        <v>496</v>
+      </c>
+      <c r="J12" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="K12" s="88"/>
+      <c r="L12" s="88"/>
+      <c r="M12" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="N12" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="O12" s="88"/>
       <c r="P12" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="Q12" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="R12" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S12" s="101" t="s">
-        <v>543</v>
-      </c>
-      <c r="T12" s="101"/>
-      <c r="U12" s="102"/>
-      <c r="V12" s="103"/>
-      <c r="W12" s="104" t="s">
+      <c r="Q12" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="R12" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S12" s="88" t="s">
+        <v>516</v>
+      </c>
+      <c r="T12" s="88"/>
+      <c r="U12" s="89"/>
+      <c r="V12" s="90"/>
+      <c r="W12" s="91" t="s">
         <v>50</v>
       </c>
     </row>
@@ -4994,46 +4973,46 @@
       <c r="E13" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="F13" s="99" t="s">
-        <v>520</v>
+      <c r="F13" s="86" t="s">
+        <v>493</v>
       </c>
       <c r="G13" s="32" t="s">
-        <v>531</v>
+        <v>504</v>
       </c>
       <c r="H13" s="32" t="s">
-        <v>532</v>
+        <v>505</v>
       </c>
       <c r="I13" s="37" t="s">
-        <v>523</v>
-      </c>
-      <c r="J13" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="K13" s="101"/>
-      <c r="L13" s="101"/>
-      <c r="M13" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="N13" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="O13" s="101"/>
+        <v>496</v>
+      </c>
+      <c r="J13" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="88"/>
+      <c r="L13" s="88"/>
+      <c r="M13" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="N13" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="O13" s="88"/>
       <c r="P13" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="Q13" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="R13" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S13" s="101" t="s">
-        <v>543</v>
-      </c>
-      <c r="T13" s="101"/>
-      <c r="U13" s="102"/>
-      <c r="V13" s="103"/>
-      <c r="W13" s="104" t="s">
+      <c r="Q13" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="R13" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S13" s="88" t="s">
+        <v>516</v>
+      </c>
+      <c r="T13" s="88"/>
+      <c r="U13" s="89"/>
+      <c r="V13" s="90"/>
+      <c r="W13" s="91" t="s">
         <v>50</v>
       </c>
     </row>
@@ -5053,46 +5032,46 @@
       <c r="E14" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="99" t="s">
-        <v>520</v>
+      <c r="F14" s="86" t="s">
+        <v>493</v>
       </c>
       <c r="G14" s="32" t="s">
-        <v>535</v>
+        <v>508</v>
       </c>
       <c r="H14" s="32" t="s">
-        <v>536</v>
+        <v>509</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>523</v>
-      </c>
-      <c r="J14" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="K14" s="101"/>
-      <c r="L14" s="101"/>
-      <c r="M14" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="N14" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="O14" s="101"/>
+        <v>496</v>
+      </c>
+      <c r="J14" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="K14" s="88"/>
+      <c r="L14" s="88"/>
+      <c r="M14" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="N14" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="O14" s="88"/>
       <c r="P14" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="Q14" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="R14" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S14" s="101" t="s">
-        <v>543</v>
-      </c>
-      <c r="T14" s="101"/>
-      <c r="U14" s="102"/>
-      <c r="V14" s="103"/>
-      <c r="W14" s="104" t="s">
+      <c r="Q14" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="R14" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S14" s="88" t="s">
+        <v>516</v>
+      </c>
+      <c r="T14" s="88"/>
+      <c r="U14" s="89"/>
+      <c r="V14" s="90"/>
+      <c r="W14" s="91" t="s">
         <v>50</v>
       </c>
     </row>
@@ -5112,46 +5091,46 @@
       <c r="E15" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="F15" s="99" t="s">
-        <v>520</v>
+      <c r="F15" s="86" t="s">
+        <v>493</v>
       </c>
       <c r="G15" s="32" t="s">
-        <v>539</v>
+        <v>512</v>
       </c>
       <c r="H15" s="32" t="s">
-        <v>540</v>
+        <v>513</v>
       </c>
       <c r="I15" s="37" t="s">
-        <v>523</v>
-      </c>
-      <c r="J15" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="K15" s="101"/>
-      <c r="L15" s="101"/>
-      <c r="M15" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="N15" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="O15" s="101"/>
+        <v>496</v>
+      </c>
+      <c r="J15" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="K15" s="88"/>
+      <c r="L15" s="88"/>
+      <c r="M15" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="N15" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="O15" s="88"/>
       <c r="P15" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="Q15" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="R15" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S15" s="101" t="s">
-        <v>543</v>
-      </c>
-      <c r="T15" s="101"/>
-      <c r="U15" s="102"/>
-      <c r="V15" s="103"/>
-      <c r="W15" s="104" t="s">
+      <c r="Q15" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="R15" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S15" s="88" t="s">
+        <v>516</v>
+      </c>
+      <c r="T15" s="88"/>
+      <c r="U15" s="89"/>
+      <c r="V15" s="90"/>
+      <c r="W15" s="91" t="s">
         <v>50</v>
       </c>
     </row>
@@ -5171,46 +5150,46 @@
       <c r="E16" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="F16" s="99" t="s">
-        <v>520</v>
+      <c r="F16" s="86" t="s">
+        <v>493</v>
       </c>
       <c r="G16" s="32" t="s">
-        <v>524</v>
+        <v>497</v>
       </c>
       <c r="H16" s="32" t="s">
-        <v>526</v>
+        <v>499</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>523</v>
-      </c>
-      <c r="J16" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="K16" s="101"/>
-      <c r="L16" s="101"/>
-      <c r="M16" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="N16" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="O16" s="101"/>
+        <v>496</v>
+      </c>
+      <c r="J16" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" s="88"/>
+      <c r="L16" s="88"/>
+      <c r="M16" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="N16" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="O16" s="88"/>
       <c r="P16" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="Q16" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="R16" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S16" s="101" t="s">
-        <v>543</v>
-      </c>
-      <c r="T16" s="101"/>
-      <c r="U16" s="102"/>
-      <c r="V16" s="103"/>
-      <c r="W16" s="104" t="s">
+      <c r="Q16" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="R16" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S16" s="88" t="s">
+        <v>516</v>
+      </c>
+      <c r="T16" s="88"/>
+      <c r="U16" s="89"/>
+      <c r="V16" s="90"/>
+      <c r="W16" s="91" t="s">
         <v>50</v>
       </c>
     </row>
@@ -5230,46 +5209,46 @@
       <c r="E17" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="99" t="s">
-        <v>520</v>
+      <c r="F17" s="86" t="s">
+        <v>493</v>
       </c>
       <c r="G17" s="32" t="s">
-        <v>529</v>
+        <v>502</v>
       </c>
       <c r="H17" s="32" t="s">
-        <v>530</v>
+        <v>503</v>
       </c>
       <c r="I17" s="37" t="s">
-        <v>523</v>
-      </c>
-      <c r="J17" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="K17" s="101"/>
-      <c r="L17" s="101"/>
-      <c r="M17" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="N17" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="O17" s="101"/>
+        <v>496</v>
+      </c>
+      <c r="J17" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="K17" s="88"/>
+      <c r="L17" s="88"/>
+      <c r="M17" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="N17" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="O17" s="88"/>
       <c r="P17" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="Q17" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="R17" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S17" s="101" t="s">
-        <v>543</v>
-      </c>
-      <c r="T17" s="101"/>
-      <c r="U17" s="102"/>
-      <c r="V17" s="103"/>
-      <c r="W17" s="104" t="s">
+      <c r="Q17" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="R17" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S17" s="88" t="s">
+        <v>516</v>
+      </c>
+      <c r="T17" s="88"/>
+      <c r="U17" s="89"/>
+      <c r="V17" s="90"/>
+      <c r="W17" s="91" t="s">
         <v>50</v>
       </c>
     </row>
@@ -5289,46 +5268,46 @@
       <c r="E18" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="F18" s="99" t="s">
-        <v>520</v>
+      <c r="F18" s="86" t="s">
+        <v>493</v>
       </c>
       <c r="G18" s="32" t="s">
-        <v>533</v>
+        <v>506</v>
       </c>
       <c r="H18" s="32" t="s">
-        <v>534</v>
+        <v>507</v>
       </c>
       <c r="I18" s="37" t="s">
-        <v>523</v>
-      </c>
-      <c r="J18" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="K18" s="101"/>
-      <c r="L18" s="101"/>
-      <c r="M18" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="N18" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="O18" s="101"/>
+        <v>496</v>
+      </c>
+      <c r="J18" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="K18" s="88"/>
+      <c r="L18" s="88"/>
+      <c r="M18" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="N18" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="O18" s="88"/>
       <c r="P18" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="Q18" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="R18" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S18" s="101" t="s">
-        <v>543</v>
-      </c>
-      <c r="T18" s="101"/>
-      <c r="U18" s="102"/>
-      <c r="V18" s="103"/>
-      <c r="W18" s="104" t="s">
+      <c r="Q18" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="R18" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S18" s="88" t="s">
+        <v>516</v>
+      </c>
+      <c r="T18" s="88"/>
+      <c r="U18" s="89"/>
+      <c r="V18" s="90"/>
+      <c r="W18" s="91" t="s">
         <v>50</v>
       </c>
     </row>
@@ -5348,46 +5327,46 @@
       <c r="E19" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="F19" s="99" t="s">
-        <v>520</v>
+      <c r="F19" s="86" t="s">
+        <v>493</v>
       </c>
       <c r="G19" s="32" t="s">
-        <v>537</v>
+        <v>510</v>
       </c>
       <c r="H19" s="32" t="s">
-        <v>538</v>
+        <v>511</v>
       </c>
       <c r="I19" s="37" t="s">
-        <v>523</v>
-      </c>
-      <c r="J19" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="K19" s="101"/>
-      <c r="L19" s="101"/>
-      <c r="M19" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="N19" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="O19" s="101"/>
+        <v>496</v>
+      </c>
+      <c r="J19" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="K19" s="88"/>
+      <c r="L19" s="88"/>
+      <c r="M19" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="N19" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="O19" s="88"/>
       <c r="P19" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="Q19" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="R19" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S19" s="101" t="s">
-        <v>543</v>
-      </c>
-      <c r="T19" s="101"/>
-      <c r="U19" s="102"/>
-      <c r="V19" s="103"/>
-      <c r="W19" s="104" t="s">
+      <c r="Q19" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="R19" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S19" s="88" t="s">
+        <v>516</v>
+      </c>
+      <c r="T19" s="88"/>
+      <c r="U19" s="89"/>
+      <c r="V19" s="90"/>
+      <c r="W19" s="91" t="s">
         <v>50</v>
       </c>
     </row>
@@ -5407,46 +5386,46 @@
       <c r="E20" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="F20" s="99" t="s">
-        <v>520</v>
+      <c r="F20" s="86" t="s">
+        <v>493</v>
       </c>
       <c r="G20" s="32" t="s">
-        <v>541</v>
+        <v>514</v>
       </c>
       <c r="H20" s="32" t="s">
-        <v>542</v>
+        <v>515</v>
       </c>
       <c r="I20" s="37" t="s">
-        <v>523</v>
-      </c>
-      <c r="J20" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="K20" s="101"/>
-      <c r="L20" s="101"/>
-      <c r="M20" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="N20" s="101" t="s">
-        <v>264</v>
-      </c>
-      <c r="O20" s="101"/>
+        <v>496</v>
+      </c>
+      <c r="J20" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="K20" s="88"/>
+      <c r="L20" s="88"/>
+      <c r="M20" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="N20" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="O20" s="88"/>
       <c r="P20" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="Q20" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="R20" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S20" s="101" t="s">
-        <v>543</v>
-      </c>
-      <c r="T20" s="101"/>
-      <c r="U20" s="102"/>
-      <c r="V20" s="103"/>
-      <c r="W20" s="104" t="s">
+      <c r="Q20" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="R20" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S20" s="88" t="s">
+        <v>516</v>
+      </c>
+      <c r="T20" s="88"/>
+      <c r="U20" s="89"/>
+      <c r="V20" s="90"/>
+      <c r="W20" s="91" t="s">
         <v>50</v>
       </c>
     </row>
@@ -5475,26 +5454,26 @@
       </c>
       <c r="K21" s="33"/>
       <c r="L21" s="33"/>
-      <c r="M21" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="N21" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="O21" s="106" t="s">
-        <v>544</v>
-      </c>
-      <c r="P21" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q21" s="106" t="s">
-        <v>264</v>
-      </c>
-      <c r="R21" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="S21" s="106" t="s">
-        <v>543</v>
+      <c r="M21" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="N21" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="O21" s="93" t="s">
+        <v>517</v>
+      </c>
+      <c r="P21" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q21" s="93" t="s">
+        <v>264</v>
+      </c>
+      <c r="R21" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="S21" s="93" t="s">
+        <v>516</v>
       </c>
       <c r="T21" s="33"/>
       <c r="U21" s="34" t="s">
@@ -5521,7 +5500,7 @@
       <c r="E22" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="F22" s="97"/>
+      <c r="F22" s="84"/>
       <c r="G22" s="32"/>
       <c r="H22" s="32"/>
       <c r="I22" s="37"/>
@@ -5530,32 +5509,32 @@
       </c>
       <c r="K22" s="33"/>
       <c r="L22" s="33"/>
-      <c r="M22" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="N22" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="O22" s="106" t="s">
-        <v>544</v>
-      </c>
-      <c r="P22" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q22" s="106" t="s">
-        <v>264</v>
-      </c>
-      <c r="R22" s="106" t="s">
+      <c r="M22" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="N22" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="O22" s="93" t="s">
+        <v>517</v>
+      </c>
+      <c r="P22" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q22" s="93" t="s">
+        <v>264</v>
+      </c>
+      <c r="R22" s="93" t="s">
         <v>67</v>
       </c>
       <c r="S22" s="43" t="s">
         <v>266</v>
       </c>
       <c r="T22" s="43"/>
-      <c r="U22" s="84" t="s">
-        <v>474</v>
-      </c>
-      <c r="V22" s="83"/>
+      <c r="U22" s="83" t="s">
+        <v>454</v>
+      </c>
+      <c r="V22" s="82"/>
       <c r="W22" s="57" t="s">
         <v>50</v>
       </c>
@@ -5576,7 +5555,7 @@
       <c r="E23" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="F23" s="97"/>
+      <c r="F23" s="84"/>
       <c r="G23" s="32"/>
       <c r="H23" s="32"/>
       <c r="I23" s="37"/>
@@ -5585,32 +5564,32 @@
       </c>
       <c r="K23" s="33"/>
       <c r="L23" s="33"/>
-      <c r="M23" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="N23" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="O23" s="106" t="s">
-        <v>544</v>
-      </c>
-      <c r="P23" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q23" s="106" t="s">
-        <v>264</v>
-      </c>
-      <c r="R23" s="106" t="s">
+      <c r="M23" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="N23" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="O23" s="93" t="s">
+        <v>517</v>
+      </c>
+      <c r="P23" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q23" s="93" t="s">
+        <v>264</v>
+      </c>
+      <c r="R23" s="93" t="s">
         <v>67</v>
       </c>
       <c r="S23" s="43" t="s">
         <v>266</v>
       </c>
       <c r="T23" s="43"/>
-      <c r="U23" s="84" t="s">
-        <v>474</v>
-      </c>
-      <c r="V23" s="83"/>
+      <c r="U23" s="83" t="s">
+        <v>454</v>
+      </c>
+      <c r="V23" s="82"/>
       <c r="W23" s="57" t="s">
         <v>50</v>
       </c>
@@ -5631,7 +5610,7 @@
       <c r="E24" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="F24" s="97"/>
+      <c r="F24" s="84"/>
       <c r="G24" s="32"/>
       <c r="H24" s="32"/>
       <c r="I24" s="37"/>
@@ -5640,32 +5619,32 @@
       </c>
       <c r="K24" s="33"/>
       <c r="L24" s="33"/>
-      <c r="M24" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="N24" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="O24" s="106" t="s">
-        <v>544</v>
-      </c>
-      <c r="P24" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q24" s="106" t="s">
-        <v>264</v>
-      </c>
-      <c r="R24" s="106" t="s">
+      <c r="M24" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="N24" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="O24" s="93" t="s">
+        <v>517</v>
+      </c>
+      <c r="P24" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q24" s="93" t="s">
+        <v>264</v>
+      </c>
+      <c r="R24" s="93" t="s">
         <v>67</v>
       </c>
       <c r="S24" s="43" t="s">
         <v>266</v>
       </c>
       <c r="T24" s="43"/>
-      <c r="U24" s="98" t="s">
-        <v>67</v>
-      </c>
-      <c r="V24" s="83"/>
+      <c r="U24" s="85" t="s">
+        <v>67</v>
+      </c>
+      <c r="V24" s="82"/>
       <c r="W24" s="57" t="s">
         <v>50</v>
       </c>
@@ -5695,32 +5674,32 @@
       </c>
       <c r="K25" s="33"/>
       <c r="L25" s="33"/>
-      <c r="M25" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="N25" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="O25" s="106" t="s">
-        <v>544</v>
-      </c>
-      <c r="P25" s="106" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q25" s="106" t="s">
-        <v>264</v>
-      </c>
-      <c r="R25" s="106" t="s">
+      <c r="M25" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="N25" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="O25" s="93" t="s">
+        <v>517</v>
+      </c>
+      <c r="P25" s="93" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q25" s="93" t="s">
+        <v>264</v>
+      </c>
+      <c r="R25" s="93" t="s">
         <v>67</v>
       </c>
       <c r="S25" s="43" t="s">
         <v>266</v>
       </c>
       <c r="T25" s="43"/>
-      <c r="U25" s="84" t="s">
-        <v>474</v>
-      </c>
-      <c r="V25" s="83"/>
+      <c r="U25" s="83" t="s">
+        <v>454</v>
+      </c>
+      <c r="V25" s="82"/>
       <c r="W25" s="57" t="s">
         <v>50</v>
       </c>
@@ -5741,22 +5720,22 @@
       <c r="E26" s="65" t="s">
         <v>73</v>
       </c>
-      <c r="F26" s="79">
+      <c r="F26" s="78">
         <v>46099</v>
       </c>
       <c r="G26" s="66" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="H26" s="67" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="I26" s="68" t="s">
-        <v>394</v>
-      </c>
-      <c r="J26" s="80" t="s">
-        <v>67</v>
-      </c>
-      <c r="K26" s="75"/>
+        <v>382</v>
+      </c>
+      <c r="J26" s="79" t="s">
+        <v>67</v>
+      </c>
+      <c r="K26" s="74"/>
       <c r="L26" s="33"/>
       <c r="M26" s="43" t="s">
         <v>264</v>
@@ -5775,7 +5754,7 @@
         <v>67</v>
       </c>
       <c r="S26" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T26" s="33"/>
       <c r="U26" s="34"/>
@@ -5800,22 +5779,22 @@
       <c r="E27" s="65" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="81">
+      <c r="F27" s="80">
         <v>46099</v>
       </c>
       <c r="G27" s="71" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="H27" s="72" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="I27" s="73" t="s">
-        <v>397</v>
-      </c>
-      <c r="J27" s="82" t="s">
-        <v>67</v>
-      </c>
-      <c r="K27" s="75"/>
+        <v>385</v>
+      </c>
+      <c r="J27" s="81" t="s">
+        <v>67</v>
+      </c>
+      <c r="K27" s="74"/>
       <c r="L27" s="33"/>
       <c r="M27" s="43" t="s">
         <v>264</v>
@@ -5834,7 +5813,7 @@
         <v>67</v>
       </c>
       <c r="S27" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T27" s="33"/>
       <c r="U27" s="34"/>
@@ -5863,13 +5842,13 @@
         <v>46099</v>
       </c>
       <c r="G28" s="69" t="s">
-        <v>398</v>
+        <v>386</v>
       </c>
       <c r="H28" s="45" t="s">
-        <v>399</v>
+        <v>387</v>
       </c>
       <c r="I28" s="70" t="s">
-        <v>400</v>
+        <v>388</v>
       </c>
       <c r="J28" s="51" t="s">
         <v>67</v>
@@ -5893,7 +5872,7 @@
         <v>67</v>
       </c>
       <c r="S28" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T28" s="33"/>
       <c r="U28" s="34"/>
@@ -5922,13 +5901,13 @@
         <v>46099</v>
       </c>
       <c r="G29" s="69" t="s">
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="H29" s="45" t="s">
-        <v>402</v>
+        <v>390</v>
       </c>
       <c r="I29" s="70" t="s">
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="J29" s="33" t="s">
         <v>67</v>
@@ -5952,7 +5931,7 @@
         <v>67</v>
       </c>
       <c r="S29" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T29" s="33"/>
       <c r="U29" s="34"/>
@@ -5981,13 +5960,13 @@
         <v>46099</v>
       </c>
       <c r="G30" s="69" t="s">
-        <v>404</v>
+        <v>392</v>
       </c>
       <c r="H30" s="45" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="I30" s="70" t="s">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="J30" s="33" t="s">
         <v>67</v>
@@ -6011,7 +5990,7 @@
         <v>67</v>
       </c>
       <c r="S30" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T30" s="33"/>
       <c r="U30" s="34"/>
@@ -6040,13 +6019,13 @@
         <v>46099</v>
       </c>
       <c r="G31" s="69" t="s">
-        <v>407</v>
+        <v>395</v>
       </c>
       <c r="H31" s="45" t="s">
-        <v>408</v>
+        <v>396</v>
       </c>
       <c r="I31" s="70" t="s">
-        <v>409</v>
+        <v>397</v>
       </c>
       <c r="J31" s="33" t="s">
         <v>67</v>
@@ -6070,7 +6049,7 @@
         <v>67</v>
       </c>
       <c r="S31" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T31" s="33"/>
       <c r="U31" s="34"/>
@@ -6099,13 +6078,13 @@
         <v>46099</v>
       </c>
       <c r="G32" s="69" t="s">
-        <v>410</v>
+        <v>398</v>
       </c>
       <c r="H32" s="45" t="s">
-        <v>411</v>
+        <v>399</v>
       </c>
       <c r="I32" s="70" t="s">
-        <v>412</v>
+        <v>400</v>
       </c>
       <c r="J32" s="33" t="s">
         <v>67</v>
@@ -6129,7 +6108,7 @@
         <v>67</v>
       </c>
       <c r="S32" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T32" s="33"/>
       <c r="U32" s="34"/>
@@ -6158,13 +6137,13 @@
         <v>46099</v>
       </c>
       <c r="G33" s="71" t="s">
-        <v>413</v>
+        <v>401</v>
       </c>
       <c r="H33" s="72" t="s">
-        <v>414</v>
+        <v>402</v>
       </c>
       <c r="I33" s="73" t="s">
-        <v>415</v>
+        <v>403</v>
       </c>
       <c r="J33" s="33" t="s">
         <v>67</v>
@@ -6188,7 +6167,7 @@
         <v>67</v>
       </c>
       <c r="S33" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T33" s="33"/>
       <c r="U33" s="34"/>
@@ -6217,13 +6196,13 @@
         <v>46099</v>
       </c>
       <c r="G34" s="56" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="H34" s="56" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="I34" s="56" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="J34" s="33" t="s">
         <v>67</v>
@@ -6247,7 +6226,7 @@
         <v>67</v>
       </c>
       <c r="S34" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T34" s="33"/>
       <c r="U34" s="34"/>
@@ -6276,13 +6255,13 @@
         <v>46099</v>
       </c>
       <c r="G35" s="45" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="H35" s="45" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="I35" s="45" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="J35" s="33" t="s">
         <v>67</v>
@@ -6306,7 +6285,7 @@
         <v>67</v>
       </c>
       <c r="S35" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T35" s="33"/>
       <c r="U35" s="34"/>
@@ -6335,13 +6314,13 @@
         <v>46099</v>
       </c>
       <c r="G36" s="45" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="H36" s="45" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="I36" s="45" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="J36" s="33" t="s">
         <v>67</v>
@@ -6365,7 +6344,7 @@
         <v>67</v>
       </c>
       <c r="S36" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T36" s="33"/>
       <c r="U36" s="34"/>
@@ -6394,13 +6373,13 @@
         <v>46099</v>
       </c>
       <c r="G37" s="45" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="H37" s="45" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="I37" s="45" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="J37" s="33" t="s">
         <v>67</v>
@@ -6424,7 +6403,7 @@
         <v>67</v>
       </c>
       <c r="S37" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T37" s="33"/>
       <c r="U37" s="34"/>
@@ -6453,13 +6432,13 @@
         <v>46099</v>
       </c>
       <c r="G38" s="45" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="H38" s="45" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="I38" s="45" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="J38" s="33" t="s">
         <v>67</v>
@@ -6483,7 +6462,7 @@
         <v>67</v>
       </c>
       <c r="S38" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T38" s="33"/>
       <c r="U38" s="34"/>
@@ -6512,13 +6491,13 @@
         <v>46099</v>
       </c>
       <c r="G39" s="45" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="H39" s="45" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
       <c r="I39" s="45" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="J39" s="33" t="s">
         <v>67</v>
@@ -6542,7 +6521,7 @@
         <v>67</v>
       </c>
       <c r="S39" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T39" s="33"/>
       <c r="U39" s="34"/>
@@ -6571,13 +6550,13 @@
         <v>46099</v>
       </c>
       <c r="G40" s="45" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="H40" s="45" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="I40" s="45" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="J40" s="33" t="s">
         <v>67</v>
@@ -6601,7 +6580,7 @@
         <v>67</v>
       </c>
       <c r="S40" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T40" s="33"/>
       <c r="U40" s="34"/>
@@ -6630,13 +6609,13 @@
         <v>46099</v>
       </c>
       <c r="G41" s="45" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
       <c r="H41" s="45" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="I41" s="45" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
       <c r="J41" s="33" t="s">
         <v>67</v>
@@ -6660,7 +6639,7 @@
         <v>67</v>
       </c>
       <c r="S41" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T41" s="33"/>
       <c r="U41" s="34"/>
@@ -6689,13 +6668,13 @@
         <v>46099</v>
       </c>
       <c r="G42" s="45" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="H42" s="45" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="I42" s="45" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="J42" s="33" t="s">
         <v>67</v>
@@ -6719,7 +6698,7 @@
         <v>67</v>
       </c>
       <c r="S42" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T42" s="33"/>
       <c r="U42" s="34"/>
@@ -6748,13 +6727,13 @@
         <v>46099</v>
       </c>
       <c r="G43" s="45" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="H43" s="45" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="I43" s="45" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="J43" s="33" t="s">
         <v>67</v>
@@ -6778,7 +6757,7 @@
         <v>67</v>
       </c>
       <c r="S43" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T43" s="33"/>
       <c r="U43" s="34"/>
@@ -6807,13 +6786,13 @@
         <v>46099</v>
       </c>
       <c r="G44" s="45" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="H44" s="45" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
       <c r="I44" s="45" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="J44" s="33" t="s">
         <v>67</v>
@@ -6837,7 +6816,7 @@
         <v>67</v>
       </c>
       <c r="S44" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T44" s="33"/>
       <c r="U44" s="34"/>
@@ -6866,13 +6845,13 @@
         <v>46099</v>
       </c>
       <c r="G45" s="45" t="s">
-        <v>365</v>
+        <v>359</v>
       </c>
       <c r="H45" s="45" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="I45" s="45" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
       <c r="J45" s="33" t="s">
         <v>67</v>
@@ -6896,7 +6875,7 @@
         <v>67</v>
       </c>
       <c r="S45" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T45" s="33"/>
       <c r="U45" s="34"/>
@@ -6925,13 +6904,13 @@
         <v>46099</v>
       </c>
       <c r="G46" s="45" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="H46" s="45" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
       <c r="I46" s="45" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="J46" s="33" t="s">
         <v>67</v>
@@ -6955,7 +6934,7 @@
         <v>67</v>
       </c>
       <c r="S46" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T46" s="33"/>
       <c r="U46" s="34"/>
@@ -6984,13 +6963,13 @@
         <v>46099</v>
       </c>
       <c r="G47" s="45" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="H47" s="45" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="I47" s="45" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
       <c r="J47" s="33" t="s">
         <v>67</v>
@@ -7014,7 +6993,7 @@
         <v>67</v>
       </c>
       <c r="S47" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T47" s="33"/>
       <c r="U47" s="34"/>
@@ -7043,13 +7022,13 @@
         <v>46099</v>
       </c>
       <c r="G48" s="45" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="H48" s="45" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
       <c r="I48" s="45" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="J48" s="33" t="s">
         <v>67</v>
@@ -7073,7 +7052,7 @@
         <v>67</v>
       </c>
       <c r="S48" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T48" s="33"/>
       <c r="U48" s="34"/>
@@ -7102,13 +7081,13 @@
         <v>46099</v>
       </c>
       <c r="G49" s="60" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="H49" s="60" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="I49" s="60" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="J49" s="33" t="s">
         <v>67</v>
@@ -7132,7 +7111,7 @@
         <v>67</v>
       </c>
       <c r="S49" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T49" s="33"/>
       <c r="U49" s="34"/>
@@ -7157,17 +7136,17 @@
       <c r="E50" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="F50" s="97" t="s">
-        <v>475</v>
+      <c r="F50" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G50" s="45" t="s">
-        <v>476</v>
+        <v>456</v>
       </c>
       <c r="H50" s="45" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
       <c r="I50" s="45" t="s">
-        <v>478</v>
+        <v>458</v>
       </c>
       <c r="J50" s="33" t="s">
         <v>67</v>
@@ -7191,7 +7170,7 @@
         <v>67</v>
       </c>
       <c r="S50" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T50" s="33"/>
       <c r="U50" s="34"/>
@@ -7216,17 +7195,17 @@
       <c r="E51" s="38" t="s">
         <v>123</v>
       </c>
-      <c r="F51" s="97" t="s">
-        <v>475</v>
+      <c r="F51" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G51" s="45" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
       <c r="H51" s="45" t="s">
-        <v>480</v>
+        <v>460</v>
       </c>
       <c r="I51" s="45" t="s">
-        <v>481</v>
+        <v>461</v>
       </c>
       <c r="J51" s="33" t="s">
         <v>67</v>
@@ -7250,7 +7229,7 @@
         <v>67</v>
       </c>
       <c r="S51" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T51" s="33"/>
       <c r="U51" s="34"/>
@@ -7275,17 +7254,17 @@
       <c r="E52" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="F52" s="97" t="s">
-        <v>475</v>
+      <c r="F52" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G52" s="45" t="s">
-        <v>482</v>
+        <v>462</v>
       </c>
       <c r="H52" s="45" t="s">
-        <v>483</v>
+        <v>463</v>
       </c>
       <c r="I52" s="45" t="s">
-        <v>484</v>
+        <v>464</v>
       </c>
       <c r="J52" s="33" t="s">
         <v>67</v>
@@ -7309,7 +7288,7 @@
         <v>67</v>
       </c>
       <c r="S52" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T52" s="33"/>
       <c r="U52" s="34"/>
@@ -7334,17 +7313,17 @@
       <c r="E53" s="38" t="s">
         <v>127</v>
       </c>
-      <c r="F53" s="97" t="s">
-        <v>475</v>
+      <c r="F53" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G53" s="45" t="s">
-        <v>485</v>
+        <v>465</v>
       </c>
       <c r="H53" s="45" t="s">
-        <v>486</v>
+        <v>466</v>
       </c>
       <c r="I53" s="45" t="s">
-        <v>487</v>
+        <v>467</v>
       </c>
       <c r="J53" s="33" t="s">
         <v>67</v>
@@ -7368,7 +7347,7 @@
         <v>67</v>
       </c>
       <c r="S53" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T53" s="33"/>
       <c r="U53" s="34"/>
@@ -7393,17 +7372,17 @@
       <c r="E54" s="38" t="s">
         <v>129</v>
       </c>
-      <c r="F54" s="97" t="s">
-        <v>475</v>
+      <c r="F54" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G54" s="45" t="s">
-        <v>488</v>
+        <v>468</v>
       </c>
       <c r="H54" s="45" t="s">
-        <v>489</v>
+        <v>469</v>
       </c>
       <c r="I54" s="45" t="s">
-        <v>490</v>
+        <v>470</v>
       </c>
       <c r="J54" s="33" t="s">
         <v>67</v>
@@ -7427,7 +7406,7 @@
         <v>67</v>
       </c>
       <c r="S54" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T54" s="33"/>
       <c r="U54" s="34"/>
@@ -7452,17 +7431,17 @@
       <c r="E55" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="F55" s="97" t="s">
-        <v>475</v>
+      <c r="F55" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G55" s="45" t="s">
-        <v>491</v>
+        <v>471</v>
       </c>
       <c r="H55" s="45" t="s">
-        <v>492</v>
+        <v>472</v>
       </c>
       <c r="I55" s="45" t="s">
-        <v>493</v>
+        <v>473</v>
       </c>
       <c r="J55" s="33" t="s">
         <v>67</v>
@@ -7486,7 +7465,7 @@
         <v>67</v>
       </c>
       <c r="S55" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T55" s="33"/>
       <c r="U55" s="34"/>
@@ -7511,17 +7490,17 @@
       <c r="E56" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="F56" s="97" t="s">
+      <c r="F56" s="84" t="s">
+        <v>455</v>
+      </c>
+      <c r="G56" s="45" t="s">
+        <v>474</v>
+      </c>
+      <c r="H56" s="45" t="s">
         <v>475</v>
       </c>
-      <c r="G56" s="45" t="s">
-        <v>494</v>
-      </c>
-      <c r="H56" s="45" t="s">
-        <v>495</v>
-      </c>
       <c r="I56" s="45" t="s">
-        <v>496</v>
+        <v>476</v>
       </c>
       <c r="J56" s="33" t="s">
         <v>67</v>
@@ -7545,7 +7524,7 @@
         <v>67</v>
       </c>
       <c r="S56" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T56" s="33"/>
       <c r="U56" s="34"/>
@@ -7570,17 +7549,17 @@
       <c r="E57" s="38" t="s">
         <v>135</v>
       </c>
-      <c r="F57" s="97" t="s">
-        <v>475</v>
+      <c r="F57" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G57" s="45" t="s">
-        <v>497</v>
+        <v>477</v>
       </c>
       <c r="H57" s="45" t="s">
-        <v>498</v>
+        <v>478</v>
       </c>
       <c r="I57" s="45" t="s">
-        <v>499</v>
+        <v>479</v>
       </c>
       <c r="J57" s="33" t="s">
         <v>67</v>
@@ -7604,7 +7583,7 @@
         <v>67</v>
       </c>
       <c r="S57" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T57" s="33"/>
       <c r="U57" s="34"/>
@@ -7629,17 +7608,17 @@
       <c r="E58" s="38" t="s">
         <v>137</v>
       </c>
-      <c r="F58" s="97" t="s">
-        <v>475</v>
+      <c r="F58" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G58" s="45" t="s">
-        <v>500</v>
+        <v>480</v>
       </c>
       <c r="H58" s="45" t="s">
-        <v>501</v>
+        <v>481</v>
       </c>
       <c r="I58" s="45" t="s">
-        <v>502</v>
+        <v>482</v>
       </c>
       <c r="J58" s="33" t="s">
         <v>67</v>
@@ -7663,7 +7642,7 @@
         <v>67</v>
       </c>
       <c r="S58" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T58" s="33"/>
       <c r="U58" s="34"/>
@@ -7688,17 +7667,17 @@
       <c r="E59" s="38" t="s">
         <v>139</v>
       </c>
-      <c r="F59" s="97" t="s">
-        <v>475</v>
+      <c r="F59" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G59" s="45" t="s">
-        <v>503</v>
+        <v>483</v>
       </c>
       <c r="H59" s="45" t="s">
-        <v>504</v>
+        <v>484</v>
       </c>
       <c r="I59" s="45" t="s">
-        <v>505</v>
+        <v>485</v>
       </c>
       <c r="J59" s="33" t="s">
         <v>67</v>
@@ -7722,7 +7701,7 @@
         <v>67</v>
       </c>
       <c r="S59" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T59" s="33"/>
       <c r="U59" s="34"/>
@@ -7747,17 +7726,17 @@
       <c r="E60" s="38" t="s">
         <v>141</v>
       </c>
-      <c r="F60" s="97" t="s">
-        <v>475</v>
+      <c r="F60" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G60" s="45" t="s">
-        <v>506</v>
+        <v>486</v>
       </c>
       <c r="H60" s="45" t="s">
-        <v>507</v>
+        <v>487</v>
       </c>
       <c r="I60" s="45" t="s">
-        <v>508</v>
+        <v>488</v>
       </c>
       <c r="J60" s="33" t="s">
         <v>67</v>
@@ -7781,7 +7760,7 @@
         <v>67</v>
       </c>
       <c r="S60" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T60" s="33"/>
       <c r="U60" s="34"/>
@@ -7810,13 +7789,13 @@
         <v>46100</v>
       </c>
       <c r="G61" s="45" t="s">
-        <v>432</v>
+        <v>412</v>
       </c>
       <c r="H61" s="45" t="s">
-        <v>433</v>
+        <v>413</v>
       </c>
       <c r="I61" s="45" t="s">
-        <v>434</v>
+        <v>414</v>
       </c>
       <c r="J61" s="33" t="s">
         <v>67</v>
@@ -7840,7 +7819,7 @@
         <v>67</v>
       </c>
       <c r="S61" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T61" s="33"/>
       <c r="U61" s="34"/>
@@ -7869,13 +7848,13 @@
         <v>46100</v>
       </c>
       <c r="G62" s="45" t="s">
-        <v>435</v>
+        <v>415</v>
       </c>
       <c r="H62" s="45" t="s">
-        <v>436</v>
+        <v>416</v>
       </c>
       <c r="I62" s="45" t="s">
-        <v>437</v>
+        <v>417</v>
       </c>
       <c r="J62" s="33" t="s">
         <v>67</v>
@@ -7899,7 +7878,7 @@
         <v>67</v>
       </c>
       <c r="S62" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T62" s="33"/>
       <c r="U62" s="34"/>
@@ -7928,13 +7907,13 @@
         <v>46100</v>
       </c>
       <c r="G63" s="45" t="s">
-        <v>438</v>
+        <v>418</v>
       </c>
       <c r="H63" s="45" t="s">
-        <v>439</v>
+        <v>419</v>
       </c>
       <c r="I63" s="45" t="s">
-        <v>440</v>
+        <v>420</v>
       </c>
       <c r="J63" s="33" t="s">
         <v>67</v>
@@ -7958,7 +7937,7 @@
         <v>67</v>
       </c>
       <c r="S63" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T63" s="33"/>
       <c r="U63" s="34"/>
@@ -7987,13 +7966,13 @@
         <v>46100</v>
       </c>
       <c r="G64" s="45" t="s">
-        <v>441</v>
+        <v>421</v>
       </c>
       <c r="H64" s="45" t="s">
-        <v>442</v>
+        <v>422</v>
       </c>
       <c r="I64" s="45" t="s">
-        <v>443</v>
+        <v>423</v>
       </c>
       <c r="J64" s="33" t="s">
         <v>67</v>
@@ -8017,7 +7996,7 @@
         <v>67</v>
       </c>
       <c r="S64" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T64" s="33"/>
       <c r="U64" s="34"/>
@@ -8046,13 +8025,13 @@
         <v>46100</v>
       </c>
       <c r="G65" s="45" t="s">
-        <v>444</v>
+        <v>424</v>
       </c>
       <c r="H65" s="45" t="s">
-        <v>445</v>
+        <v>425</v>
       </c>
       <c r="I65" s="45" t="s">
-        <v>446</v>
+        <v>426</v>
       </c>
       <c r="J65" s="33" t="s">
         <v>67</v>
@@ -8076,7 +8055,7 @@
         <v>67</v>
       </c>
       <c r="S65" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T65" s="33"/>
       <c r="U65" s="34"/>
@@ -8105,13 +8084,13 @@
         <v>46100</v>
       </c>
       <c r="G66" s="45" t="s">
-        <v>447</v>
+        <v>427</v>
       </c>
       <c r="H66" s="45" t="s">
-        <v>448</v>
+        <v>428</v>
       </c>
       <c r="I66" s="45" t="s">
-        <v>449</v>
+        <v>429</v>
       </c>
       <c r="J66" s="33" t="s">
         <v>67</v>
@@ -8135,7 +8114,7 @@
         <v>67</v>
       </c>
       <c r="S66" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T66" s="33"/>
       <c r="U66" s="34"/>
@@ -8164,13 +8143,13 @@
         <v>46100</v>
       </c>
       <c r="G67" s="45" t="s">
-        <v>450</v>
+        <v>430</v>
       </c>
       <c r="H67" s="45" t="s">
-        <v>451</v>
+        <v>431</v>
       </c>
       <c r="I67" s="45" t="s">
-        <v>452</v>
+        <v>432</v>
       </c>
       <c r="J67" s="33" t="s">
         <v>67</v>
@@ -8194,7 +8173,7 @@
         <v>67</v>
       </c>
       <c r="S67" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T67" s="33"/>
       <c r="U67" s="34"/>
@@ -8223,13 +8202,13 @@
         <v>46100</v>
       </c>
       <c r="G68" s="45" t="s">
-        <v>453</v>
+        <v>433</v>
       </c>
       <c r="H68" s="45" t="s">
-        <v>454</v>
+        <v>434</v>
       </c>
       <c r="I68" s="45" t="s">
-        <v>455</v>
+        <v>435</v>
       </c>
       <c r="J68" s="33" t="s">
         <v>67</v>
@@ -8253,7 +8232,7 @@
         <v>67</v>
       </c>
       <c r="S68" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T68" s="33"/>
       <c r="U68" s="34"/>
@@ -8282,13 +8261,13 @@
         <v>46100</v>
       </c>
       <c r="G69" s="45" t="s">
-        <v>456</v>
+        <v>436</v>
       </c>
       <c r="H69" s="45" t="s">
-        <v>457</v>
+        <v>437</v>
       </c>
       <c r="I69" s="45" t="s">
-        <v>458</v>
+        <v>438</v>
       </c>
       <c r="J69" s="33" t="s">
         <v>67</v>
@@ -8312,7 +8291,7 @@
         <v>67</v>
       </c>
       <c r="S69" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T69" s="33"/>
       <c r="U69" s="34"/>
@@ -8341,13 +8320,13 @@
         <v>46100</v>
       </c>
       <c r="G70" s="45" t="s">
-        <v>459</v>
+        <v>439</v>
       </c>
       <c r="H70" s="45" t="s">
-        <v>460</v>
+        <v>440</v>
       </c>
       <c r="I70" s="45" t="s">
-        <v>461</v>
+        <v>441</v>
       </c>
       <c r="J70" s="33" t="s">
         <v>67</v>
@@ -8371,7 +8350,7 @@
         <v>67</v>
       </c>
       <c r="S70" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T70" s="33"/>
       <c r="U70" s="34"/>
@@ -8400,13 +8379,13 @@
         <v>46100</v>
       </c>
       <c r="G71" s="45" t="s">
-        <v>462</v>
+        <v>442</v>
       </c>
       <c r="H71" s="45" t="s">
-        <v>463</v>
+        <v>443</v>
       </c>
       <c r="I71" s="45" t="s">
-        <v>464</v>
+        <v>444</v>
       </c>
       <c r="J71" s="33" t="s">
         <v>67</v>
@@ -8430,7 +8409,7 @@
         <v>67</v>
       </c>
       <c r="S71" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T71" s="33"/>
       <c r="U71" s="34"/>
@@ -8459,13 +8438,13 @@
         <v>46100</v>
       </c>
       <c r="G72" s="45" t="s">
-        <v>465</v>
+        <v>445</v>
       </c>
       <c r="H72" s="45" t="s">
-        <v>466</v>
+        <v>446</v>
       </c>
       <c r="I72" s="45" t="s">
-        <v>467</v>
+        <v>447</v>
       </c>
       <c r="J72" s="33" t="s">
         <v>67</v>
@@ -8489,7 +8468,7 @@
         <v>67</v>
       </c>
       <c r="S72" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T72" s="33"/>
       <c r="U72" s="34"/>
@@ -8518,13 +8497,13 @@
         <v>46100</v>
       </c>
       <c r="G73" s="45" t="s">
-        <v>468</v>
+        <v>448</v>
       </c>
       <c r="H73" s="45" t="s">
-        <v>469</v>
+        <v>449</v>
       </c>
       <c r="I73" s="45" t="s">
-        <v>470</v>
+        <v>450</v>
       </c>
       <c r="J73" s="33" t="s">
         <v>67</v>
@@ -8548,7 +8527,7 @@
         <v>67</v>
       </c>
       <c r="S73" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T73" s="33"/>
       <c r="U73" s="34"/>
@@ -8603,11 +8582,11 @@
       <c r="Q74" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R74" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S74" s="101" t="s">
-        <v>543</v>
+      <c r="R74" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S74" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T74" s="33"/>
       <c r="U74" s="34"/>
@@ -8662,11 +8641,11 @@
       <c r="Q75" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R75" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S75" s="101" t="s">
-        <v>543</v>
+      <c r="R75" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S75" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T75" s="33"/>
       <c r="U75" s="34"/>
@@ -8721,11 +8700,11 @@
       <c r="Q76" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R76" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S76" s="101" t="s">
-        <v>543</v>
+      <c r="R76" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S76" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T76" s="33"/>
       <c r="U76" s="34"/>
@@ -8780,11 +8759,11 @@
       <c r="Q77" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R77" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S77" s="101" t="s">
-        <v>543</v>
+      <c r="R77" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S77" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T77" s="33"/>
       <c r="U77" s="34"/>
@@ -8839,11 +8818,11 @@
       <c r="Q78" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R78" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S78" s="101" t="s">
-        <v>543</v>
+      <c r="R78" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S78" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T78" s="33"/>
       <c r="U78" s="34"/>
@@ -8898,11 +8877,11 @@
       <c r="Q79" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R79" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S79" s="101" t="s">
-        <v>543</v>
+      <c r="R79" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S79" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T79" s="33"/>
       <c r="U79" s="34"/>
@@ -8957,11 +8936,11 @@
       <c r="Q80" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R80" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S80" s="101" t="s">
-        <v>543</v>
+      <c r="R80" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S80" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T80" s="33"/>
       <c r="U80" s="34"/>
@@ -9016,11 +8995,11 @@
       <c r="Q81" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R81" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S81" s="101" t="s">
-        <v>543</v>
+      <c r="R81" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S81" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T81" s="33"/>
       <c r="U81" s="34"/>
@@ -9075,11 +9054,11 @@
       <c r="Q82" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R82" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S82" s="101" t="s">
-        <v>543</v>
+      <c r="R82" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S82" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T82" s="33"/>
       <c r="U82" s="34"/>
@@ -9134,11 +9113,11 @@
       <c r="Q83" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R83" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S83" s="101" t="s">
-        <v>543</v>
+      <c r="R83" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S83" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T83" s="33"/>
       <c r="U83" s="34"/>
@@ -9193,11 +9172,11 @@
       <c r="Q84" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R84" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S84" s="101" t="s">
-        <v>543</v>
+      <c r="R84" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S84" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T84" s="33"/>
       <c r="U84" s="34"/>
@@ -9252,11 +9231,11 @@
       <c r="Q85" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R85" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S85" s="101" t="s">
-        <v>543</v>
+      <c r="R85" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S85" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T85" s="33"/>
       <c r="U85" s="34"/>
@@ -9311,11 +9290,11 @@
       <c r="Q86" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R86" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S86" s="101" t="s">
-        <v>543</v>
+      <c r="R86" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S86" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T86" s="33"/>
       <c r="U86" s="34"/>
@@ -9370,11 +9349,11 @@
       <c r="Q87" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R87" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S87" s="101" t="s">
-        <v>543</v>
+      <c r="R87" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S87" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T87" s="33"/>
       <c r="U87" s="34"/>
@@ -9429,11 +9408,11 @@
       <c r="Q88" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R88" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S88" s="101" t="s">
-        <v>543</v>
+      <c r="R88" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S88" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T88" s="33"/>
       <c r="U88" s="34"/>
@@ -9443,7 +9422,7 @@
       </c>
     </row>
     <row r="89" spans="1:23" ht="135.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="105">
+      <c r="A89" s="92">
         <v>191</v>
       </c>
       <c r="B89" s="31" t="s">
@@ -9462,14 +9441,14 @@
       <c r="G89" s="32"/>
       <c r="H89" s="32"/>
       <c r="I89" s="37"/>
-      <c r="J89" s="107" t="s">
-        <v>264</v>
-      </c>
-      <c r="K89" s="108" t="s">
+      <c r="J89" s="94" t="s">
+        <v>264</v>
+      </c>
+      <c r="K89" s="95" t="s">
         <v>245</v>
       </c>
-      <c r="L89" s="107" t="s">
-        <v>545</v>
+      <c r="L89" s="94" t="s">
+        <v>518</v>
       </c>
       <c r="M89" s="33"/>
       <c r="N89" s="33"/>
@@ -9486,7 +9465,7 @@
       </c>
     </row>
     <row r="90" spans="1:23" ht="135.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="105">
+      <c r="A90" s="92">
         <v>376</v>
       </c>
       <c r="B90" s="31" t="s">
@@ -9505,14 +9484,14 @@
       <c r="G90" s="32"/>
       <c r="H90" s="32"/>
       <c r="I90" s="37"/>
-      <c r="J90" s="109" t="s">
-        <v>264</v>
-      </c>
-      <c r="K90" s="110" t="s">
+      <c r="J90" s="94" t="s">
+        <v>264</v>
+      </c>
+      <c r="K90" s="95" t="s">
         <v>245</v>
       </c>
-      <c r="L90" s="109" t="s">
-        <v>545</v>
+      <c r="L90" s="94" t="s">
+        <v>518</v>
       </c>
       <c r="M90" s="33"/>
       <c r="N90" s="33"/>
@@ -9545,16 +9524,16 @@
         <v>203</v>
       </c>
       <c r="F91" s="44">
-        <v>46098</v>
+        <v>46111</v>
       </c>
       <c r="G91" s="45" t="s">
-        <v>317</v>
+        <v>527</v>
       </c>
       <c r="H91" s="45" t="s">
-        <v>318</v>
+        <v>519</v>
       </c>
       <c r="I91" s="45" t="s">
-        <v>319</v>
+        <v>520</v>
       </c>
       <c r="J91" s="33" t="s">
         <v>67</v>
@@ -9592,16 +9571,16 @@
         <v>205</v>
       </c>
       <c r="F92" s="44">
-        <v>46098</v>
+        <v>46111</v>
       </c>
       <c r="G92" s="45" t="s">
-        <v>320</v>
+        <v>528</v>
       </c>
       <c r="H92" s="45" t="s">
-        <v>321</v>
+        <v>522</v>
       </c>
       <c r="I92" s="45" t="s">
-        <v>322</v>
+        <v>521</v>
       </c>
       <c r="J92" s="33" t="s">
         <v>67</v>
@@ -9638,17 +9617,17 @@
       <c r="E93" s="65" t="s">
         <v>207</v>
       </c>
-      <c r="F93" s="74">
-        <v>46099</v>
+      <c r="F93" s="44">
+        <v>46111</v>
       </c>
       <c r="G93" s="45" t="s">
-        <v>416</v>
+        <v>531</v>
       </c>
       <c r="H93" s="45" t="s">
-        <v>417</v>
+        <v>532</v>
       </c>
       <c r="I93" s="45" t="s">
-        <v>418</v>
+        <v>533</v>
       </c>
       <c r="J93" s="33" t="s">
         <v>67</v>
@@ -9689,13 +9668,13 @@
         <v>46099</v>
       </c>
       <c r="G94" s="45" t="s">
-        <v>519</v>
+        <v>492</v>
       </c>
       <c r="H94" s="45" t="s">
-        <v>428</v>
+        <v>410</v>
       </c>
       <c r="I94" s="45" t="s">
-        <v>429</v>
+        <v>411</v>
       </c>
       <c r="J94" s="33" t="s">
         <v>67</v>
@@ -9733,16 +9712,16 @@
         <v>211</v>
       </c>
       <c r="F95" s="44">
-        <v>46099</v>
+        <v>46112</v>
       </c>
       <c r="G95" s="45" t="s">
-        <v>509</v>
+        <v>541</v>
       </c>
       <c r="H95" s="45" t="s">
-        <v>430</v>
+        <v>537</v>
       </c>
       <c r="I95" s="45" t="s">
-        <v>431</v>
+        <v>538</v>
       </c>
       <c r="J95" s="33" t="s">
         <v>67</v>
@@ -9779,17 +9758,17 @@
       <c r="E96" s="38" t="s">
         <v>213</v>
       </c>
-      <c r="F96" s="97" t="s">
-        <v>475</v>
+      <c r="F96" s="84" t="s">
+        <v>539</v>
       </c>
       <c r="G96" s="45" t="s">
-        <v>510</v>
+        <v>540</v>
       </c>
       <c r="H96" s="45" t="s">
-        <v>511</v>
+        <v>542</v>
       </c>
       <c r="I96" s="45" t="s">
-        <v>512</v>
+        <v>543</v>
       </c>
       <c r="J96" s="33" t="s">
         <v>67</v>
@@ -9826,17 +9805,17 @@
       <c r="E97" s="38" t="s">
         <v>215</v>
       </c>
-      <c r="F97" s="97" t="s">
-        <v>475</v>
+      <c r="F97" s="84" t="s">
+        <v>539</v>
       </c>
       <c r="G97" s="45" t="s">
-        <v>513</v>
+        <v>544</v>
       </c>
       <c r="H97" s="45" t="s">
-        <v>514</v>
+        <v>545</v>
       </c>
       <c r="I97" s="45" t="s">
-        <v>515</v>
+        <v>546</v>
       </c>
       <c r="J97" s="33" t="s">
         <v>67</v>
@@ -9877,13 +9856,13 @@
         <v>46098</v>
       </c>
       <c r="G98" s="45" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="H98" s="45" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="I98" s="45" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="J98" s="33" t="s">
         <v>67</v>
@@ -9903,11 +9882,11 @@
       <c r="Q98" s="49" t="s">
         <v>316</v>
       </c>
-      <c r="R98" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S98" s="101" t="s">
-        <v>543</v>
+      <c r="R98" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S98" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T98" s="33"/>
       <c r="U98" s="34"/>
@@ -9936,13 +9915,13 @@
         <v>46099</v>
       </c>
       <c r="G99" s="64" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="H99" s="64" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="I99" s="64" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="J99" s="33" t="s">
         <v>67</v>
@@ -9966,7 +9945,7 @@
         <v>67</v>
       </c>
       <c r="S99" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T99" s="33"/>
       <c r="U99" s="34"/>
@@ -9991,17 +9970,17 @@
       <c r="E100" s="38" t="s">
         <v>221</v>
       </c>
-      <c r="F100" s="97" t="s">
-        <v>475</v>
+      <c r="F100" s="84" t="s">
+        <v>455</v>
       </c>
       <c r="G100" s="45" t="s">
-        <v>516</v>
+        <v>489</v>
       </c>
       <c r="H100" s="45" t="s">
-        <v>517</v>
+        <v>490</v>
       </c>
       <c r="I100" s="45" t="s">
-        <v>518</v>
+        <v>491</v>
       </c>
       <c r="J100" s="33" t="s">
         <v>67</v>
@@ -10025,7 +10004,7 @@
         <v>67</v>
       </c>
       <c r="S100" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T100" s="33"/>
       <c r="U100" s="34"/>
@@ -10054,13 +10033,13 @@
         <v>46100</v>
       </c>
       <c r="G101" s="45" t="s">
-        <v>471</v>
+        <v>451</v>
       </c>
       <c r="H101" s="45" t="s">
-        <v>472</v>
+        <v>452</v>
       </c>
       <c r="I101" s="45" t="s">
-        <v>473</v>
+        <v>453</v>
       </c>
       <c r="J101" s="33" t="s">
         <v>67</v>
@@ -10084,7 +10063,7 @@
         <v>67</v>
       </c>
       <c r="S101" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T101" s="33"/>
       <c r="U101" s="34"/>
@@ -10113,13 +10092,13 @@
         <v>46099</v>
       </c>
       <c r="G102" s="45" t="s">
-        <v>422</v>
+        <v>404</v>
       </c>
       <c r="H102" s="45" t="s">
-        <v>423</v>
+        <v>405</v>
       </c>
       <c r="I102" s="45" t="s">
-        <v>424</v>
+        <v>406</v>
       </c>
       <c r="J102" s="33" t="s">
         <v>67</v>
@@ -10143,7 +10122,7 @@
         <v>67</v>
       </c>
       <c r="S102" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T102" s="33"/>
       <c r="U102" s="34"/>
@@ -10172,13 +10151,13 @@
         <v>46098</v>
       </c>
       <c r="G103" s="45" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="H103" s="45" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="I103" s="45" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="J103" s="33" t="s">
         <v>67</v>
@@ -10198,11 +10177,11 @@
       <c r="Q103" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="R103" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S103" s="101" t="s">
-        <v>543</v>
+      <c r="R103" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S103" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T103" s="33"/>
       <c r="U103" s="34"/>
@@ -10227,17 +10206,17 @@
       <c r="E104" s="38" t="s">
         <v>229</v>
       </c>
-      <c r="F104" s="55">
-        <v>46099</v>
+      <c r="F104" s="59">
+        <v>46111</v>
       </c>
       <c r="G104" s="56" t="s">
-        <v>383</v>
+        <v>529</v>
       </c>
       <c r="H104" s="56" t="s">
-        <v>384</v>
+        <v>524</v>
       </c>
       <c r="I104" s="56" t="s">
-        <v>385</v>
+        <v>523</v>
       </c>
       <c r="J104" s="33" t="s">
         <v>67</v>
@@ -10275,16 +10254,16 @@
         <v>231</v>
       </c>
       <c r="F105" s="59">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="G105" s="60" t="s">
-        <v>386</v>
+        <v>530</v>
       </c>
       <c r="H105" s="60" t="s">
-        <v>387</v>
+        <v>525</v>
       </c>
       <c r="I105" s="60" t="s">
-        <v>388</v>
+        <v>526</v>
       </c>
       <c r="J105" s="33" t="s">
         <v>67</v>
@@ -10325,13 +10304,13 @@
         <v>46099</v>
       </c>
       <c r="G106" s="45" t="s">
-        <v>425</v>
+        <v>407</v>
       </c>
       <c r="H106" s="45" t="s">
-        <v>426</v>
+        <v>408</v>
       </c>
       <c r="I106" s="45" t="s">
-        <v>427</v>
+        <v>409</v>
       </c>
       <c r="J106" s="33" t="s">
         <v>67</v>
@@ -10355,7 +10334,7 @@
         <v>67</v>
       </c>
       <c r="S106" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T106" s="33"/>
       <c r="U106" s="34"/>
@@ -10384,13 +10363,13 @@
         <v>46099</v>
       </c>
       <c r="G107" s="64" t="s">
-        <v>389</v>
+        <v>377</v>
       </c>
       <c r="H107" s="64" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="I107" s="64" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="J107" s="33" t="s">
         <v>67</v>
@@ -10414,7 +10393,7 @@
         <v>67</v>
       </c>
       <c r="S107" s="33" t="s">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="T107" s="33"/>
       <c r="U107" s="34"/>
@@ -10443,13 +10422,13 @@
         <v>46098</v>
       </c>
       <c r="G108" s="53" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="H108" s="45" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="I108" s="45" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="J108" s="33" t="s">
         <v>67</v>
@@ -10469,11 +10448,11 @@
       <c r="Q108" s="54" t="s">
         <v>316</v>
       </c>
-      <c r="R108" s="101" t="s">
-        <v>67</v>
-      </c>
-      <c r="S108" s="101" t="s">
-        <v>543</v>
+      <c r="R108" s="88" t="s">
+        <v>67</v>
+      </c>
+      <c r="S108" s="88" t="s">
+        <v>516</v>
       </c>
       <c r="T108" s="33"/>
       <c r="U108" s="34"/>
@@ -13475,7 +13454,7 @@
   <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="3">
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{F5F4AC7B-142E-4F14-AD0B-95E75DB6B433}">
           <x14:formula1>
             <xm:f>Sheet1!$B$2:$B$3</xm:f>
@@ -15651,6 +15630,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
@@ -15660,15 +15648,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -15936,6 +15915,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
@@ -15948,14 +15935,6 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Aggiornamento file pdf per case test non superati
CN: A1#111#CENTROBIОЛABSERVICE
subject_application_id:CBS POLIAMBULATORIO	
subject_application_vendor:CENTRO BIOLAB SERVICE SRL	
subject_application_version:1.57

Aggiornamento file pdf per case test non superati 4, 457, 458, 459, 471, 472
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#CENTROBIOLABSERVICE/CENTRO_BIOLAB_SERVICE_SRL/CBS_POLIAMBULATORIO/1.57/report-checklist.xlsx
+++ b/GATEWAY/A1#111#CENTROBIOLABSERVICE/CENTRO_BIOLAB_SERVICE_SRL/CBS_POLIAMBULATORIO/1.57/report-checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paolo\OneDrive\Desktop\FSE Puglia\accreditamento fse git\ESITO TESTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0FD102C-3170-475C-A502-0659C7FD1BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{249AC4A9-9A66-4160-B120-3A84ECC317F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1937,30 +1937,12 @@
     <t>704f665ed66c5cbcd6df451b38e22efa</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.8fe46b71d98546dc779f4a7f4859b056b254bbe56b59baa550333b2c46441c87.8ec86adcd6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>52e94d7170f4b0182ad993cf69b9f173</t>
-  </si>
-  <si>
-    <t>39fc441612ab744470c1ad3026939989</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.8fe46b71d98546dc779f4a7f4859b056b254bbe56b59baa550333b2c46441c87.0c9feae58a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-03-30T18:02:22Z</t>
   </si>
   <si>
     <t>2026-03-30T18:25:58Z</t>
   </si>
   <si>
-    <t>2026-03-30T18:29:21Z</t>
-  </si>
-  <si>
-    <t>2026-03-30T18:32:37Z</t>
-  </si>
-  <si>
     <t>2026-03-30T16:19:03Z</t>
   </si>
   <si>
@@ -1970,43 +1952,61 @@
     <t>2.16.840.1.113883.2.9.2.120.4.4.97bb3fc5bee3032679f4f07419e04af6375baafa17024527a98ede920c6812ed.7402ea81d8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>ca5a49210d49663ee4e2b46baf363443</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.97bb3fc5bee3032679f4f07419e04af6375baafa17024527a98ede920c6812ed.778f52725e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-31T08:46:27Z</t>
-  </si>
-  <si>
-    <t>9b0b68160dafc70938db708407790326</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.40d0883912^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>31/03/2026</t>
   </si>
   <si>
-    <t>2026-03-31T09:03:46Z</t>
-  </si>
-  <si>
-    <t>2026-03-31T08:59:56Z</t>
-  </si>
-  <si>
-    <t>804c39bdfb45649a7a0198638da4fa2a</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.8ea47d33ac^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-31T09:08:30Z</t>
-  </si>
-  <si>
-    <t>e2ac9ee378eed70710d429e673992b50</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.b5ff942f15^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.97bb3fc5bee3032679f4f07419e04af6375baafa17024527a98ede920c6812ed.dd425d1533^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>bfb2c0d84a94ba8f4a2cdb34d4b40d11</t>
+  </si>
+  <si>
+    <t>2026-03-31T18:03:53Z</t>
+  </si>
+  <si>
+    <t>9110742debcb3abfed56e9973b88fccd</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.8fe46b71d98546dc779f4a7f4859b056b254bbe56b59baa550333b2c46441c87.6ba6e125b1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-31T18:11:48Z</t>
+  </si>
+  <si>
+    <t>2026-03-31T18:16:57Z</t>
+  </si>
+  <si>
+    <t>0e315901cf9d60d876c54e2dd5e477df</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.8fe46b71d98546dc779f4a7f4859b056b254bbe56b59baa550333b2c46441c87.98444447c9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-31T18:39:01Z</t>
+  </si>
+  <si>
+    <t>04eb22c980538a1ff3905eb0268bc804</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.b1ad185ea1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-31T18:47:28Z</t>
+  </si>
+  <si>
+    <t>c456934afc3d80642cee3cc261aecf95</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.f183d1f2f7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-31T18:50:43Z</t>
+  </si>
+  <si>
+    <t>85383f86e3ad4e617c8df5c2c9c9c6d1</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.bedba6cc08^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -2016,11 +2016,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2753,136 +2760,136 @@
   </borders>
   <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2891,22 +2898,22 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2945,7 +2952,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2972,10 +2979,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -2987,78 +2994,87 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -4812,13 +4828,13 @@
         <v>46112</v>
       </c>
       <c r="G10" s="77" t="s">
-        <v>536</v>
+        <v>531</v>
       </c>
       <c r="H10" s="77" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="I10" s="77" t="s">
-        <v>535</v>
+        <v>529</v>
       </c>
       <c r="J10" s="79" t="s">
         <v>67</v>
@@ -9527,7 +9543,7 @@
         <v>46111</v>
       </c>
       <c r="G91" s="45" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="H91" s="45" t="s">
         <v>519</v>
@@ -9574,7 +9590,7 @@
         <v>46111</v>
       </c>
       <c r="G92" s="45" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="H92" s="45" t="s">
         <v>522</v>
@@ -9621,13 +9637,13 @@
         <v>46111</v>
       </c>
       <c r="G93" s="45" t="s">
-        <v>531</v>
+        <v>525</v>
       </c>
       <c r="H93" s="45" t="s">
-        <v>532</v>
+        <v>526</v>
       </c>
       <c r="I93" s="45" t="s">
-        <v>533</v>
+        <v>527</v>
       </c>
       <c r="J93" s="33" t="s">
         <v>67</v>
@@ -9715,13 +9731,13 @@
         <v>46112</v>
       </c>
       <c r="G95" s="45" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="H95" s="45" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="I95" s="45" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="J95" s="33" t="s">
         <v>67</v>
@@ -9759,10 +9775,10 @@
         <v>213</v>
       </c>
       <c r="F96" s="84" t="s">
-        <v>539</v>
+        <v>528</v>
       </c>
       <c r="G96" s="45" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="H96" s="45" t="s">
         <v>542</v>
@@ -9806,7 +9822,7 @@
         <v>215</v>
       </c>
       <c r="F97" s="84" t="s">
-        <v>539</v>
+        <v>528</v>
       </c>
       <c r="G97" s="45" t="s">
         <v>544</v>
@@ -10207,16 +10223,16 @@
         <v>229</v>
       </c>
       <c r="F104" s="59">
-        <v>46111</v>
-      </c>
-      <c r="G104" s="56" t="s">
-        <v>529</v>
+        <v>46112</v>
+      </c>
+      <c r="G104" s="108" t="s">
+        <v>534</v>
       </c>
       <c r="H104" s="56" t="s">
-        <v>524</v>
-      </c>
-      <c r="I104" s="56" t="s">
-        <v>523</v>
+        <v>532</v>
+      </c>
+      <c r="I104" s="108" t="s">
+        <v>533</v>
       </c>
       <c r="J104" s="33" t="s">
         <v>67</v>
@@ -10254,16 +10270,16 @@
         <v>231</v>
       </c>
       <c r="F105" s="59">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="G105" s="60" t="s">
-        <v>530</v>
-      </c>
-      <c r="H105" s="60" t="s">
-        <v>525</v>
-      </c>
-      <c r="I105" s="60" t="s">
-        <v>526</v>
+        <v>535</v>
+      </c>
+      <c r="H105" s="109" t="s">
+        <v>536</v>
+      </c>
+      <c r="I105" s="110" t="s">
+        <v>537</v>
       </c>
       <c r="J105" s="33" t="s">
         <v>67</v>
@@ -13448,13 +13464,13 @@
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
   </mergeCells>
-  <phoneticPr fontId="17" type="noConversion"/>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{F5F4AC7B-142E-4F14-AD0B-95E75DB6B433}">
           <x14:formula1>
             <xm:f>Sheet1!$B$2:$B$3</xm:f>

</xml_diff>

<commit_message>
Aggiornamento file PDF test case non superati
CN: A1#111#CENTROBIОЛABSERVICE
subject_application_id:CBS POLIAMBULATORIO	
subject_application_vendor:CENTRO BIOLAB SERVICE SRL	
subject_application_version:1.57

Aggiornamento file PDF test case non superati 457 458 459
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#CENTROBIOLABSERVICE/CENTRO_BIOLAB_SERVICE_SRL/CBS_POLIAMBULATORIO/1.57/report-checklist.xlsx
+++ b/GATEWAY/A1#111#CENTROBIOLABSERVICE/CENTRO_BIOLAB_SERVICE_SRL/CBS_POLIAMBULATORIO/1.57/report-checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paolo\OneDrive\Desktop\FSE Puglia\accreditamento fse git\ESITO TESTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{249AC4A9-9A66-4160-B120-3A84ECC317F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9E57A2-A0C5-417D-9756-69B923073471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="547">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="546">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -1952,9 +1952,6 @@
     <t>2.16.840.1.113883.2.9.2.120.4.4.97bb3fc5bee3032679f4f07419e04af6375baafa17024527a98ede920c6812ed.7402ea81d8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>31/03/2026</t>
-  </si>
-  <si>
     <t>2.16.840.1.113883.2.9.2.120.4.4.97bb3fc5bee3032679f4f07419e04af6375baafa17024527a98ede920c6812ed.dd425d1533^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
@@ -1982,31 +1979,31 @@
     <t>2.16.840.1.113883.2.9.2.120.4.4.8fe46b71d98546dc779f4a7f4859b056b254bbe56b59baa550333b2c46441c87.98444447c9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>2026-03-31T18:39:01Z</t>
-  </si>
-  <si>
-    <t>04eb22c980538a1ff3905eb0268bc804</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.b1ad185ea1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-31T18:47:28Z</t>
-  </si>
-  <si>
-    <t>c456934afc3d80642cee3cc261aecf95</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.f183d1f2f7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-31T18:50:43Z</t>
-  </si>
-  <si>
-    <t>85383f86e3ad4e617c8df5c2c9c9c6d1</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.bedba6cc08^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>219542524d6149afa1fc23cbba1a91ba</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.18276cff84^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-04-01T18:58:08Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.aaab26600e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>c3c6abe880ea893ad8e580c67a7548f3</t>
+  </si>
+  <si>
+    <t>2026-04-01T19:04:07Z</t>
+  </si>
+  <si>
+    <t>2026-04-01T19:06:50Z</t>
+  </si>
+  <si>
+    <t>0b8a096931182f34fa67c898ade591c2</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.d07b8a7c92^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -3045,6 +3042,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3066,15 +3072,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -4563,14 +4560,14 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="98" t="s">
+      <c r="A2" s="101" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="99"/>
-      <c r="C2" s="100" t="s">
+      <c r="B2" s="102"/>
+      <c r="C2" s="103" t="s">
         <v>267</v>
       </c>
-      <c r="D2" s="99"/>
+      <c r="D2" s="102"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -4591,14 +4588,14 @@
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="104" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="107" t="s">
+      <c r="B3" s="105"/>
+      <c r="C3" s="110" t="s">
         <v>268</v>
       </c>
-      <c r="D3" s="99"/>
+      <c r="D3" s="102"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -4619,12 +4616,12 @@
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="103"/>
-      <c r="B4" s="104"/>
-      <c r="C4" s="107" t="s">
+      <c r="A4" s="106"/>
+      <c r="B4" s="107"/>
+      <c r="C4" s="110" t="s">
         <v>269</v>
       </c>
-      <c r="D4" s="99"/>
+      <c r="D4" s="102"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -4646,12 +4643,12 @@
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="105"/>
-      <c r="B5" s="106"/>
-      <c r="C5" s="107" t="s">
+      <c r="A5" s="108"/>
+      <c r="B5" s="109"/>
+      <c r="C5" s="110" t="s">
         <v>270</v>
       </c>
-      <c r="D5" s="99"/>
+      <c r="D5" s="102"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -4672,8 +4669,8 @@
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="96"/>
-      <c r="B6" s="97"/>
+      <c r="A6" s="99"/>
+      <c r="B6" s="100"/>
       <c r="C6" s="10"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -4828,13 +4825,13 @@
         <v>46112</v>
       </c>
       <c r="G10" s="77" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H10" s="77" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="I10" s="77" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="J10" s="79" t="s">
         <v>67</v>
@@ -9728,16 +9725,16 @@
         <v>211</v>
       </c>
       <c r="F95" s="44">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="G95" s="45" t="s">
+        <v>539</v>
+      </c>
+      <c r="H95" s="45" t="s">
+        <v>537</v>
+      </c>
+      <c r="I95" s="45" t="s">
         <v>538</v>
-      </c>
-      <c r="H95" s="45" t="s">
-        <v>539</v>
-      </c>
-      <c r="I95" s="45" t="s">
-        <v>540</v>
       </c>
       <c r="J95" s="33" t="s">
         <v>67</v>
@@ -9774,17 +9771,17 @@
       <c r="E96" s="38" t="s">
         <v>213</v>
       </c>
-      <c r="F96" s="84" t="s">
-        <v>528</v>
+      <c r="F96" s="44">
+        <v>46113</v>
       </c>
       <c r="G96" s="45" t="s">
+        <v>542</v>
+      </c>
+      <c r="H96" s="45" t="s">
         <v>541</v>
       </c>
-      <c r="H96" s="45" t="s">
-        <v>542</v>
-      </c>
       <c r="I96" s="45" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="J96" s="33" t="s">
         <v>67</v>
@@ -9821,17 +9818,17 @@
       <c r="E97" s="38" t="s">
         <v>215</v>
       </c>
-      <c r="F97" s="84" t="s">
-        <v>528</v>
+      <c r="F97" s="44">
+        <v>46113</v>
       </c>
       <c r="G97" s="45" t="s">
+        <v>543</v>
+      </c>
+      <c r="H97" s="45" t="s">
         <v>544</v>
       </c>
-      <c r="H97" s="45" t="s">
+      <c r="I97" s="45" t="s">
         <v>545</v>
-      </c>
-      <c r="I97" s="45" t="s">
-        <v>546</v>
       </c>
       <c r="J97" s="33" t="s">
         <v>67</v>
@@ -10225,14 +10222,14 @@
       <c r="F104" s="59">
         <v>46112</v>
       </c>
-      <c r="G104" s="108" t="s">
-        <v>534</v>
+      <c r="G104" s="96" t="s">
+        <v>533</v>
       </c>
       <c r="H104" s="56" t="s">
+        <v>531</v>
+      </c>
+      <c r="I104" s="96" t="s">
         <v>532</v>
-      </c>
-      <c r="I104" s="108" t="s">
-        <v>533</v>
       </c>
       <c r="J104" s="33" t="s">
         <v>67</v>
@@ -10273,13 +10270,13 @@
         <v>46112</v>
       </c>
       <c r="G105" s="60" t="s">
+        <v>534</v>
+      </c>
+      <c r="H105" s="97" t="s">
         <v>535</v>
       </c>
-      <c r="H105" s="109" t="s">
+      <c r="I105" s="98" t="s">
         <v>536</v>
-      </c>
-      <c r="I105" s="110" t="s">
-        <v>537</v>
       </c>
       <c r="J105" s="33" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Centro Biolab Services - Aggiornamento
CN: A1#111#CENTROBIОЛABSERVICE
subject_application_id:CBS POLIAMBULATORIO	
subject_application_vendor:CENTRO BIOLAB SERVICE SRL	
subject_application_version:1.57
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#CENTROBIOLABSERVICE/CENTRO_BIOLAB_SERVICE_SRL/CBS_POLIAMBULATORIO/1.57/report-checklist.xlsx
+++ b/GATEWAY/A1#111#CENTROBIOLABSERVICE/CENTRO_BIOLAB_SERVICE_SRL/CBS_POLIAMBULATORIO/1.57/report-checklist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paolo\OneDrive\Desktop\FSE Puglia\accreditamento fse git\ESITO TESTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9E57A2-A0C5-417D-9756-69B923073471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C27507-D10D-42ED-8E20-477CD029B6D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1997,13 +1997,13 @@
     <t>2026-04-01T19:04:07Z</t>
   </si>
   <si>
-    <t>2026-04-01T19:06:50Z</t>
-  </si>
-  <si>
-    <t>0b8a096931182f34fa67c898ade591c2</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.d07b8a7c92^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-07T19:25:19Z</t>
+  </si>
+  <si>
+    <t>19a4df0dfab9a9290fb9429b0d8cf2f2</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.46a41df0ab0514f11c0811056832c3225e06c8e11824f27c7e5517ca5cfc57fe.2970d36689^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -2013,11 +2013,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2757,136 +2764,136 @@
   </borders>
   <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2895,22 +2902,22 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2949,7 +2956,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2976,10 +2983,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -2991,87 +2998,90 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -9819,7 +9829,7 @@
         <v>215</v>
       </c>
       <c r="F97" s="44">
-        <v>46113</v>
+        <v>46119</v>
       </c>
       <c r="G97" s="45" t="s">
         <v>543</v>
@@ -9827,7 +9837,7 @@
       <c r="H97" s="45" t="s">
         <v>544</v>
       </c>
-      <c r="I97" s="45" t="s">
+      <c r="I97" s="111" t="s">
         <v>545</v>
       </c>
       <c r="J97" s="33" t="s">
@@ -13461,7 +13471,7 @@
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
   </mergeCells>
-  <phoneticPr fontId="18" type="noConversion"/>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
@@ -15643,15 +15653,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
@@ -15661,6 +15662,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -15928,14 +15938,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
@@ -15948,6 +15950,14 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>